<commit_message>
Added imaginary vessel performance
</commit_message>
<xml_diff>
--- a/modelado/modelos/resultados/Class/DL_cla.xlsx
+++ b/modelado/modelos/resultados/Class/DL_cla.xlsx
@@ -3,32 +3,37 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="UNet3D_SQA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="UNet3D_HKP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="StackedCNN3D_SQA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="StackedCNN3D_HKP" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CNN3D_SQA" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CNN3D_HKP" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CNN3D_SQA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CNN3D_HKP" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="UNet3D_SQA_todas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="UNet3D_HKP_todas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,12 +47,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -60,9 +80,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -153,7 +176,7 @@
     <ext cx="9420225" cy="2847975"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -163,7 +186,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -181,7 +206,7 @@
     <ext cx="8096250" cy="2990850"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPr id="3" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -191,7 +216,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -209,7 +236,7 @@
     <ext cx="6210300" cy="4667250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPr id="4" name="Image 3" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -219,7 +246,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -242,7 +271,7 @@
     <ext cx="9420225" cy="2847975"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -252,7 +281,12 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -267,7 +301,7 @@
     <ext cx="8096250" cy="2990850"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPr id="3" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -277,7 +311,12 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -292,7 +331,7 @@
     <ext cx="6210300" cy="4667250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPr id="4" name="Image 3" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -302,7 +341,12 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -322,7 +366,7 @@
     <ext cx="9420225" cy="2847975"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -332,7 +376,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -350,7 +396,7 @@
     <ext cx="8096250" cy="2990850"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPr id="3" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -360,7 +406,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -375,10 +423,10 @@
       <row>40</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6296025" cy="4667250"/>
+    <ext cx="6210300" cy="4667250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPr id="4" name="Image 3" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -388,7 +436,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -408,10 +458,10 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9420225" cy="2847975"/>
+    <ext cx="9429750" cy="2847975"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -421,7 +471,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -439,7 +491,7 @@
     <ext cx="8096250" cy="2990850"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPr id="3" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -449,7 +501,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -464,10 +518,10 @@
       <row>40</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6296025" cy="4667250"/>
+    <ext cx="6210300" cy="4667250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPr id="4" name="Image 3" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -477,7 +531,9 @@
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -586,7 +642,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9420225" cy="2847975"/>
+    <ext cx="9429750" cy="2847975"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -600,9 +656,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -628,9 +681,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -656,9 +706,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -934,7 +981,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -947,7 +994,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
@@ -1210,7 +1257,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
@@ -1473,7 +1520,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
@@ -1505,22 +1552,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.867±0.011</t>
+          <t>0.839±0.011</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.874±0.019</t>
+          <t>0.902±0.029</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.870±0.007</t>
+          <t>0.869±0.010</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3038.000±0.000</t>
+          <t>924.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1532,22 +1579,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.652±0.040</t>
+          <t>0.727±0.052</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.589±0.043</t>
+          <t>0.605±0.048</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.616±0.014</t>
+          <t>0.657±0.017</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>731.000±0.000</t>
+          <t>288.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1559,22 +1606,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.667±0.029</t>
+          <t>0.773±0.035</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.704±0.030</t>
+          <t>0.707±0.031</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.684±0.008</t>
+          <t>0.738±0.015</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>731.000±0.000</t>
+          <t>288.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1586,22 +1633,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.800±0.007</t>
+          <t>0.808±0.012</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.800±0.007</t>
+          <t>0.808±0.012</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.800±0.007</t>
+          <t>0.808±0.012</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.800±0.007</t>
+          <t>0.808±0.012</t>
         </is>
       </c>
     </row>
@@ -1613,22 +1660,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.729±0.011</t>
+          <t>0.780±0.022</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.722±0.012</t>
+          <t>0.738±0.011</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.724±0.006</t>
+          <t>0.755±0.011</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4500.000±0.000</t>
+          <t>1500.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1640,22 +1687,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.800±0.005</t>
+          <t>0.805±0.011</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.800±0.007</t>
+          <t>0.808±0.012</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.799±0.006</t>
+          <t>0.803±0.010</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4500.000±0.000</t>
+          <t>1500.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1721,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.771±0.011</t>
+          <t>0.769±0.016</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1733,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.446±0.015</t>
+          <t>0.490±0.019</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1745,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.520±0.010</t>
+          <t>0.584±0.019</t>
         </is>
       </c>
     </row>
@@ -1712,14 +1759,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0.591±0.011</t>
+          <t>0.635±0.018</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0.710±0.047</t>
+          <t>0.655±0.079</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1783,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
@@ -1768,22 +1815,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.834±0.015</t>
+          <t>0.846±0.022</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.834±0.017</t>
+          <t>0.851±0.034</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.834±0.004</t>
+          <t>0.848±0.009</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2510.000±0.000</t>
+          <t>810.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1795,22 +1842,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.467±0.020</t>
+          <t>0.515±0.031</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.381±0.031</t>
+          <t>0.368±0.030</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.419±0.023</t>
+          <t>0.427±0.013</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>995.000±0.000</t>
+          <t>345.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1822,22 +1869,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.592±0.018</t>
+          <t>0.569±0.014</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.699±0.022</t>
+          <t>0.719±0.045</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.641±0.005</t>
+          <t>0.634±0.017</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>995.000±0.000</t>
+          <t>345.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1896,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.704±0.007</t>
+          <t>0.709±0.010</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.704±0.007</t>
+          <t>0.709±0.010</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.704±0.007</t>
+          <t>0.709±0.010</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.704±0.007</t>
+          <t>0.709±0.010</t>
         </is>
       </c>
     </row>
@@ -1876,22 +1923,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.631±0.010</t>
+          <t>0.643±0.010</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.638±0.009</t>
+          <t>0.646±0.011</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.631±0.010</t>
+          <t>0.636±0.009</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4500.000±0.000</t>
+          <t>1500.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1903,22 +1950,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.699±0.008</t>
+          <t>0.706±0.009</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.704±0.007</t>
+          <t>0.709±0.010</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.699±0.007</t>
+          <t>0.702±0.008</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4500.000±0.000</t>
+          <t>1500.000±0.000</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1984,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.715±0.006</t>
+          <t>0.736±0.014</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1996,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.265±0.018</t>
+          <t>0.272±0.011</t>
         </is>
       </c>
     </row>
@@ -1961,7 +2008,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.471±0.005</t>
+          <t>0.465±0.018</t>
         </is>
       </c>
     </row>
@@ -1975,14 +2022,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0.499±0.011</t>
+          <t>0.517±0.013</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0.799±0.037</t>
+          <t>0.704±0.087</t>
         </is>
       </c>
     </row>
@@ -2002,46 +2049,46 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>f1-score</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.805±0.017</t>
+          <t>0.820±0.032</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.935±0.015</t>
+          <t>0.918±0.016</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.865±0.006</t>
+          <t>0.866±0.013</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2051,24 +2098,24 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.758±0.037</t>
+          <t>0.730±0.041</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.510±0.078</t>
+          <t>0.560±0.114</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.605±0.048</t>
+          <t>0.628±0.083</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2078,24 +2125,24 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.780±0.030</t>
+          <t>0.754±0.037</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.623±0.041</t>
+          <t>0.634±0.065</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.692±0.026</t>
+          <t>0.687±0.044</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2105,51 +2152,51 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.793±0.009</t>
+          <t>0.795±0.023</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.793±0.009</t>
+          <t>0.795±0.023</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.793±0.009</t>
+          <t>0.795±0.023</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.793±0.009</t>
+          <t>0.795±0.023</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>macro avg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.781±0.018</t>
+          <t>0.768±0.021</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.689±0.019</t>
+          <t>0.704±0.049</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.720±0.016</t>
+          <t>0.727±0.043</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2159,24 +2206,24 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>weighted avg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.791±0.010</t>
+          <t>0.790±0.024</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.793±0.009</t>
+          <t>0.795±0.023</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.781±0.012</t>
+          <t>0.786±0.030</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2186,50 +2233,50 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>IoU</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Clase 0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.762±0.009</t>
+          <t>0.764±0.020</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Clase 1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.435±0.049</t>
+          <t>0.462±0.081</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Clase 2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.529±0.032</t>
+          <t>0.525±0.051</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Mean ± Std</t>
         </is>
@@ -2238,14 +2285,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0.590±0.022</t>
+          <t>0.600±0.059</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0.474±0.090</t>
+          <t>0.497±0.208</t>
         </is>
       </c>
     </row>
@@ -2265,46 +2312,46 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>f1-score</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.825±0.022</t>
+          <t>0.841±0.014</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.877±0.025</t>
+          <t>0.867±0.012</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.850±0.007</t>
+          <t>0.854±0.009</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2314,24 +2361,24 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.500±0.040</t>
+          <t>0.485±0.028</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.365±0.043</t>
+          <t>0.391±0.031</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.418±0.020</t>
+          <t>0.431±0.014</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2341,24 +2388,24 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.584±0.013</t>
+          <t>0.575±0.010</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.648±0.058</t>
+          <t>0.642±0.058</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.613±0.026</t>
+          <t>0.605±0.026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2368,51 +2415,51 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.707±0.010</t>
+          <t>0.706±0.009</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.707±0.010</t>
+          <t>0.706±0.009</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.707±0.010</t>
+          <t>0.706±0.009</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.707±0.010</t>
+          <t>0.706±0.009</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>macro avg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.636±0.012</t>
+          <t>0.634±0.010</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.630±0.014</t>
+          <t>0.633±0.012</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.627±0.011</t>
+          <t>0.630±0.008</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2422,24 +2469,24 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>weighted avg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.695±0.011</t>
+          <t>0.698±0.010</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.707±0.010</t>
+          <t>0.706±0.009</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.696±0.008</t>
+          <t>0.699±0.008</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2449,50 +2496,50 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>IoU</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Clase 0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.739±0.011</t>
+          <t>0.745±0.014</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Clase 1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.265±0.016</t>
+          <t>0.275±0.012</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Clase 2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.443±0.027</t>
+          <t>0.435±0.026</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Mean ± Std</t>
         </is>
@@ -2501,14 +2548,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0.504±0.017</t>
+          <t>0.507±0.016</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0.803±0.055</t>
+          <t>0.819±0.039</t>
         </is>
       </c>
     </row>

</xml_diff>